<commit_message>
Add discussion to output folder and update excel sheet to be consistent across all sheets
</commit_message>
<xml_diff>
--- a/DataClustering/output_phase4/phase4_results.xlsx
+++ b/DataClustering/output_phase4/phase4_results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aiden\source\repos\DataClustering\DataClustering\output_phase4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aiden Cary\DataClustering\Data-Clustering\DataClustering\output_phase4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD92F823-3AC1-4A98-AE21-6AEF424C01F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52017680-16B5-42DF-A4C4-2BE574BBFCDE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="16515" windowHeight="14580" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="396" yWindow="396" windowWidth="16512" windowHeight="14580" firstSheet="3" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ecoli" sheetId="1" r:id="rId1"/>
@@ -23,13 +23,17 @@
     <sheet name="Vehicle" sheetId="8" r:id="rId8"/>
     <sheet name="Wine" sheetId="9" r:id="rId9"/>
     <sheet name="Yeast" sheetId="10" r:id="rId10"/>
+    <sheet name="K Estimation Summary" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="30">
+  <si>
+    <t>ecoli.txt (True K = 8)</t>
+  </si>
   <si>
     <t>K</t>
   </si>
@@ -49,7 +53,7 @@
     <t>Best Estimated K (SW):</t>
   </si>
   <si>
-    <t>True K:</t>
+    <t>True K (From Phase 2):</t>
   </si>
   <si>
     <t>glass.txt  (True K = 6)</t>
@@ -79,10 +83,43 @@
     <t>yeast.txt  (True K = 10)</t>
   </si>
   <si>
-    <t>True K (From Phase 2):</t>
+    <t>Dataset</t>
   </si>
   <si>
-    <t>ecoli.txt (True K = 8)</t>
+    <t>Best K (CH)</t>
+  </si>
+  <si>
+    <t>Best K (SW)</t>
+  </si>
+  <si>
+    <t>Ecoli</t>
+  </si>
+  <si>
+    <t>Glass</t>
+  </si>
+  <si>
+    <t>Ionosphere</t>
+  </si>
+  <si>
+    <t>Iris Bezdek</t>
+  </si>
+  <si>
+    <t>Landsat</t>
+  </si>
+  <si>
+    <t>Letter Recognition</t>
+  </si>
+  <si>
+    <t>Segmentation</t>
+  </si>
+  <si>
+    <t>Vehicle</t>
+  </si>
+  <si>
+    <t>Wine</t>
+  </si>
+  <si>
+    <t>Yeast</t>
   </si>
 </sst>
 </file>
@@ -92,7 +129,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -119,8 +156,14 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -137,6 +180,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
         <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF4472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -167,7 +222,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -188,6 +243,19 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -495,36 +563,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="1" max="1" width="22" style="8" customWidth="1"/>
+    <col min="2" max="3" width="18" style="8" customWidth="1"/>
+    <col min="4" max="4" width="12" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18.75" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -536,7 +604,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -548,7 +616,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -560,7 +628,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -572,7 +640,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -584,7 +652,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -596,7 +664,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -610,7 +678,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -622,7 +690,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -634,7 +702,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -646,7 +714,7 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -658,7 +726,7 @@
       </c>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -670,25 +738,25 @@
       </c>
       <c r="D14" s="2"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4">
       <c r="A16" s="7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B16" s="7">
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2">
       <c r="A17" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B17" s="7">
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2">
       <c r="A18" s="7" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B18" s="7">
         <v>8</v>
@@ -705,36 +773,36 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:D32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="1" max="1" width="22" style="8" customWidth="1"/>
+    <col min="2" max="3" width="18" style="8" customWidth="1"/>
+    <col min="4" max="4" width="12" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18.75" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -746,7 +814,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -758,7 +826,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -770,7 +838,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -782,7 +850,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -794,7 +862,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -806,7 +874,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -818,7 +886,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -830,7 +898,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -844,7 +912,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -856,7 +924,7 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -868,7 +936,7 @@
       </c>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -880,7 +948,7 @@
       </c>
       <c r="D14" s="2"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -892,7 +960,7 @@
       </c>
       <c r="D15" s="2"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -904,7 +972,7 @@
       </c>
       <c r="D16" s="2"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -916,7 +984,7 @@
       </c>
       <c r="D17" s="2"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -928,7 +996,7 @@
       </c>
       <c r="D18" s="2"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -940,7 +1008,7 @@
       </c>
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -952,7 +1020,7 @@
       </c>
       <c r="D20" s="2"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -964,7 +1032,7 @@
       </c>
       <c r="D21" s="2"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -976,7 +1044,7 @@
       </c>
       <c r="D22" s="2"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -988,7 +1056,7 @@
       </c>
       <c r="D23" s="2"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1000,7 +1068,7 @@
       </c>
       <c r="D24" s="2"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1012,7 +1080,7 @@
       </c>
       <c r="D25" s="2"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1024,7 +1092,7 @@
       </c>
       <c r="D26" s="2"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1036,7 +1104,7 @@
       </c>
       <c r="D27" s="2"/>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1048,25 +1116,25 @@
       </c>
       <c r="D28" s="2"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4">
       <c r="A30" s="7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B30" s="7">
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4">
       <c r="A31" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B31" s="7">
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4">
       <c r="A32" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B32" s="7">
         <v>10</v>
@@ -1080,39 +1148,209 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="22" style="8" customWidth="1"/>
+    <col min="2" max="2" width="10" style="8" customWidth="1"/>
+    <col min="3" max="4" width="14" style="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="11">
+        <v>8</v>
+      </c>
+      <c r="C2" s="11">
+        <v>4</v>
+      </c>
+      <c r="D2" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="11">
+        <v>6</v>
+      </c>
+      <c r="C3" s="11">
+        <v>2</v>
+      </c>
+      <c r="D3" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="11">
+        <v>2</v>
+      </c>
+      <c r="C4" s="12">
+        <v>2</v>
+      </c>
+      <c r="D4" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="11">
+        <v>3</v>
+      </c>
+      <c r="C5" s="12">
+        <v>3</v>
+      </c>
+      <c r="D5" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="11">
+        <v>6</v>
+      </c>
+      <c r="C6" s="11">
+        <v>3</v>
+      </c>
+      <c r="D6" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="11">
+        <v>26</v>
+      </c>
+      <c r="C7" s="11">
+        <v>2</v>
+      </c>
+      <c r="D7" s="11">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="11">
+        <v>7</v>
+      </c>
+      <c r="C8" s="11">
+        <v>4</v>
+      </c>
+      <c r="D8" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="11">
+        <v>4</v>
+      </c>
+      <c r="C9" s="11">
+        <v>2</v>
+      </c>
+      <c r="D9" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="11">
+        <v>3</v>
+      </c>
+      <c r="C10" s="11">
+        <v>2</v>
+      </c>
+      <c r="D10" s="12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="11">
+        <v>10</v>
+      </c>
+      <c r="C11" s="11">
+        <v>2</v>
+      </c>
+      <c r="D11" s="11">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="1" max="1" width="22" style="8" customWidth="1"/>
+    <col min="2" max="3" width="18" style="8" customWidth="1"/>
+    <col min="4" max="4" width="12" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18.75" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1124,7 +1362,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1136,7 +1374,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1148,7 +1386,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1160,7 +1398,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1174,7 +1412,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1186,7 +1424,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1198,7 +1436,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1210,7 +1448,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1222,25 +1460,25 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4">
       <c r="A13" s="7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B13" s="7">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4">
       <c r="A14" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B14" s="7">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4">
       <c r="A15" s="7" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B15" s="7">
         <v>6</v>
@@ -1257,36 +1495,36 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="1" max="1" width="22" style="8" customWidth="1"/>
+    <col min="2" max="3" width="18" style="8" customWidth="1"/>
+    <col min="4" max="4" width="12" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18.75" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1300,7 +1538,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1312,7 +1550,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -1324,7 +1562,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1336,7 +1574,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1348,7 +1586,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1360,7 +1598,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1372,7 +1610,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1384,7 +1622,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1396,7 +1634,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1408,7 +1646,7 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1420,7 +1658,7 @@
       </c>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1432,25 +1670,25 @@
       </c>
       <c r="D14" s="2"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4">
       <c r="A16" s="7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B16" s="7">
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2">
       <c r="A17" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B17" s="7">
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2">
       <c r="A18" s="7" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B18" s="7">
         <v>2</v>
@@ -1467,36 +1705,36 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="1" max="1" width="22" style="8" customWidth="1"/>
+    <col min="2" max="3" width="18" style="8" customWidth="1"/>
+    <col min="4" max="4" width="12" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18.75" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1508,7 +1746,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1522,7 +1760,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1534,7 +1772,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1546,7 +1784,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1558,7 +1796,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1570,7 +1808,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1582,7 +1820,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1594,25 +1832,25 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4">
       <c r="A12" s="7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B12" s="7">
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4">
       <c r="A13" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B13" s="7">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4">
       <c r="A14" s="7" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B14" s="7">
         <v>3</v>
@@ -1629,36 +1867,36 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D62"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="1" max="1" width="22" style="8" customWidth="1"/>
+    <col min="2" max="3" width="18" style="8" customWidth="1"/>
+    <col min="4" max="4" width="12" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18.75" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1670,7 +1908,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1682,7 +1920,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1694,7 +1932,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1706,7 +1944,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1720,7 +1958,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1732,7 +1970,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1744,7 +1982,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1756,7 +1994,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1768,7 +2006,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1780,7 +2018,7 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1792,7 +2030,7 @@
       </c>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1804,7 +2042,7 @@
       </c>
       <c r="D14" s="2"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1816,7 +2054,7 @@
       </c>
       <c r="D15" s="2"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1828,7 +2066,7 @@
       </c>
       <c r="D16" s="2"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1840,7 +2078,7 @@
       </c>
       <c r="D17" s="2"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1852,7 +2090,7 @@
       </c>
       <c r="D18" s="2"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1864,7 +2102,7 @@
       </c>
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1876,7 +2114,7 @@
       </c>
       <c r="D20" s="2"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1888,7 +2126,7 @@
       </c>
       <c r="D21" s="2"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1900,7 +2138,7 @@
       </c>
       <c r="D22" s="2"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1912,7 +2150,7 @@
       </c>
       <c r="D23" s="2"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1924,7 +2162,7 @@
       </c>
       <c r="D24" s="2"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1936,7 +2174,7 @@
       </c>
       <c r="D25" s="2"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1948,7 +2186,7 @@
       </c>
       <c r="D26" s="2"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1960,7 +2198,7 @@
       </c>
       <c r="D27" s="2"/>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1972,7 +2210,7 @@
       </c>
       <c r="D28" s="2"/>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -1984,7 +2222,7 @@
       </c>
       <c r="D29" s="2"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -1996,7 +2234,7 @@
       </c>
       <c r="D30" s="2"/>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -2008,7 +2246,7 @@
       </c>
       <c r="D31" s="2"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -2020,7 +2258,7 @@
       </c>
       <c r="D32" s="2"/>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -2032,7 +2270,7 @@
       </c>
       <c r="D33" s="2"/>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -2044,7 +2282,7 @@
       </c>
       <c r="D34" s="2"/>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -2056,7 +2294,7 @@
       </c>
       <c r="D35" s="2"/>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2068,7 +2306,7 @@
       </c>
       <c r="D36" s="2"/>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -2080,7 +2318,7 @@
       </c>
       <c r="D37" s="2"/>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -2092,7 +2330,7 @@
       </c>
       <c r="D38" s="2"/>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -2104,7 +2342,7 @@
       </c>
       <c r="D39" s="2"/>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -2116,7 +2354,7 @@
       </c>
       <c r="D40" s="2"/>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -2128,7 +2366,7 @@
       </c>
       <c r="D41" s="2"/>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -2140,7 +2378,7 @@
       </c>
       <c r="D42" s="2"/>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -2152,7 +2390,7 @@
       </c>
       <c r="D43" s="2"/>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -2164,7 +2402,7 @@
       </c>
       <c r="D44" s="2"/>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -2176,7 +2414,7 @@
       </c>
       <c r="D45" s="2"/>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -2188,7 +2426,7 @@
       </c>
       <c r="D46" s="2"/>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -2200,7 +2438,7 @@
       </c>
       <c r="D47" s="2"/>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -2212,7 +2450,7 @@
       </c>
       <c r="D48" s="2"/>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -2224,7 +2462,7 @@
       </c>
       <c r="D49" s="2"/>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -2236,7 +2474,7 @@
       </c>
       <c r="D50" s="2"/>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -2248,7 +2486,7 @@
       </c>
       <c r="D51" s="2"/>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -2260,7 +2498,7 @@
       </c>
       <c r="D52" s="2"/>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -2272,7 +2510,7 @@
       </c>
       <c r="D53" s="2"/>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -2284,7 +2522,7 @@
       </c>
       <c r="D54" s="2"/>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -2296,7 +2534,7 @@
       </c>
       <c r="D55" s="2"/>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -2308,7 +2546,7 @@
       </c>
       <c r="D56" s="2"/>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -2320,7 +2558,7 @@
       </c>
       <c r="D57" s="2"/>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -2332,25 +2570,25 @@
       </c>
       <c r="D58" s="2"/>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4">
       <c r="A60" s="7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B60" s="7">
         <v>3</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4">
       <c r="A61" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B61" s="7">
         <v>3</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4">
       <c r="A62" s="7" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B62" s="7">
         <v>6</v>
@@ -2367,36 +2605,36 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:D105"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="1" max="1" width="22" style="8" customWidth="1"/>
+    <col min="2" max="3" width="18" style="8" customWidth="1"/>
+    <col min="4" max="4" width="12" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18.75" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -2408,7 +2646,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -2420,7 +2658,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -2432,7 +2670,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -2444,7 +2682,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -2456,7 +2694,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -2468,7 +2706,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -2480,7 +2718,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -2492,7 +2730,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -2504,7 +2742,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -2516,7 +2754,7 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -2528,7 +2766,7 @@
       </c>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -2540,7 +2778,7 @@
       </c>
       <c r="D14" s="2"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -2552,7 +2790,7 @@
       </c>
       <c r="D15" s="2"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -2564,7 +2802,7 @@
       </c>
       <c r="D16" s="2"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -2576,7 +2814,7 @@
       </c>
       <c r="D17" s="2"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -2588,7 +2826,7 @@
       </c>
       <c r="D18" s="2"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -2600,7 +2838,7 @@
       </c>
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -2612,7 +2850,7 @@
       </c>
       <c r="D20" s="2"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -2624,7 +2862,7 @@
       </c>
       <c r="D21" s="2"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -2636,7 +2874,7 @@
       </c>
       <c r="D22" s="2"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -2648,7 +2886,7 @@
       </c>
       <c r="D23" s="2"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -2660,7 +2898,7 @@
       </c>
       <c r="D24" s="2"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -2672,7 +2910,7 @@
       </c>
       <c r="D25" s="2"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -2684,7 +2922,7 @@
       </c>
       <c r="D26" s="2"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -2698,7 +2936,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -2710,7 +2948,7 @@
       </c>
       <c r="D28" s="2"/>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -2722,7 +2960,7 @@
       </c>
       <c r="D29" s="2"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -2734,7 +2972,7 @@
       </c>
       <c r="D30" s="2"/>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -2746,7 +2984,7 @@
       </c>
       <c r="D31" s="2"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -2758,7 +2996,7 @@
       </c>
       <c r="D32" s="2"/>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -2770,7 +3008,7 @@
       </c>
       <c r="D33" s="2"/>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -2782,7 +3020,7 @@
       </c>
       <c r="D34" s="2"/>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -2794,7 +3032,7 @@
       </c>
       <c r="D35" s="2"/>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2806,7 +3044,7 @@
       </c>
       <c r="D36" s="2"/>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -2818,7 +3056,7 @@
       </c>
       <c r="D37" s="2"/>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -2830,7 +3068,7 @@
       </c>
       <c r="D38" s="2"/>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -2842,7 +3080,7 @@
       </c>
       <c r="D39" s="2"/>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -2854,7 +3092,7 @@
       </c>
       <c r="D40" s="2"/>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -2866,7 +3104,7 @@
       </c>
       <c r="D41" s="2"/>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -2878,7 +3116,7 @@
       </c>
       <c r="D42" s="2"/>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -2890,7 +3128,7 @@
       </c>
       <c r="D43" s="2"/>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -2902,7 +3140,7 @@
       </c>
       <c r="D44" s="2"/>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -2914,7 +3152,7 @@
       </c>
       <c r="D45" s="2"/>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -2926,7 +3164,7 @@
       </c>
       <c r="D46" s="2"/>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -2938,7 +3176,7 @@
       </c>
       <c r="D47" s="2"/>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -2950,7 +3188,7 @@
       </c>
       <c r="D48" s="2"/>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -2962,7 +3200,7 @@
       </c>
       <c r="D49" s="2"/>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -2974,7 +3212,7 @@
       </c>
       <c r="D50" s="2"/>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -2986,7 +3224,7 @@
       </c>
       <c r="D51" s="2"/>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -2998,7 +3236,7 @@
       </c>
       <c r="D52" s="2"/>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -3010,7 +3248,7 @@
       </c>
       <c r="D53" s="2"/>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -3022,7 +3260,7 @@
       </c>
       <c r="D54" s="2"/>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -3034,7 +3272,7 @@
       </c>
       <c r="D55" s="2"/>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -3046,7 +3284,7 @@
       </c>
       <c r="D56" s="2"/>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -3058,7 +3296,7 @@
       </c>
       <c r="D57" s="2"/>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -3070,7 +3308,7 @@
       </c>
       <c r="D58" s="2"/>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -3082,7 +3320,7 @@
       </c>
       <c r="D59" s="2"/>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -3094,7 +3332,7 @@
       </c>
       <c r="D60" s="2"/>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -3106,7 +3344,7 @@
       </c>
       <c r="D61" s="2"/>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -3118,7 +3356,7 @@
       </c>
       <c r="D62" s="2"/>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -3130,7 +3368,7 @@
       </c>
       <c r="D63" s="2"/>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -3142,7 +3380,7 @@
       </c>
       <c r="D64" s="2"/>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -3154,7 +3392,7 @@
       </c>
       <c r="D65" s="2"/>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -3166,7 +3404,7 @@
       </c>
       <c r="D66" s="2"/>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -3178,7 +3416,7 @@
       </c>
       <c r="D67" s="2"/>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -3190,7 +3428,7 @@
       </c>
       <c r="D68" s="2"/>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -3202,7 +3440,7 @@
       </c>
       <c r="D69" s="2"/>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -3214,7 +3452,7 @@
       </c>
       <c r="D70" s="2"/>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -3226,7 +3464,7 @@
       </c>
       <c r="D71" s="2"/>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -3238,7 +3476,7 @@
       </c>
       <c r="D72" s="2"/>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -3250,7 +3488,7 @@
       </c>
       <c r="D73" s="2"/>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -3262,7 +3500,7 @@
       </c>
       <c r="D74" s="2"/>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4">
       <c r="A75" s="2">
         <v>74</v>
       </c>
@@ -3274,7 +3512,7 @@
       </c>
       <c r="D75" s="2"/>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4">
       <c r="A76" s="2">
         <v>75</v>
       </c>
@@ -3286,7 +3524,7 @@
       </c>
       <c r="D76" s="2"/>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4">
       <c r="A77" s="2">
         <v>76</v>
       </c>
@@ -3298,7 +3536,7 @@
       </c>
       <c r="D77" s="2"/>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -3310,7 +3548,7 @@
       </c>
       <c r="D78" s="2"/>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -3322,7 +3560,7 @@
       </c>
       <c r="D79" s="2"/>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -3334,7 +3572,7 @@
       </c>
       <c r="D80" s="2"/>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -3346,7 +3584,7 @@
       </c>
       <c r="D81" s="2"/>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4">
       <c r="A82" s="2">
         <v>81</v>
       </c>
@@ -3358,7 +3596,7 @@
       </c>
       <c r="D82" s="2"/>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4">
       <c r="A83" s="2">
         <v>82</v>
       </c>
@@ -3370,7 +3608,7 @@
       </c>
       <c r="D83" s="2"/>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4">
       <c r="A84" s="2">
         <v>83</v>
       </c>
@@ -3382,7 +3620,7 @@
       </c>
       <c r="D84" s="2"/>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -3394,7 +3632,7 @@
       </c>
       <c r="D85" s="2"/>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4">
       <c r="A86" s="4">
         <v>85</v>
       </c>
@@ -3406,7 +3644,7 @@
       </c>
       <c r="D86" s="2"/>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -3418,7 +3656,7 @@
       </c>
       <c r="D87" s="2"/>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -3430,7 +3668,7 @@
       </c>
       <c r="D88" s="2"/>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -3442,7 +3680,7 @@
       </c>
       <c r="D89" s="2"/>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -3454,7 +3692,7 @@
       </c>
       <c r="D90" s="2"/>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -3466,7 +3704,7 @@
       </c>
       <c r="D91" s="2"/>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -3478,7 +3716,7 @@
       </c>
       <c r="D92" s="2"/>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -3490,7 +3728,7 @@
       </c>
       <c r="D93" s="2"/>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4">
       <c r="A94" s="2">
         <v>93</v>
       </c>
@@ -3502,7 +3740,7 @@
       </c>
       <c r="D94" s="2"/>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4">
       <c r="A95" s="2">
         <v>94</v>
       </c>
@@ -3514,7 +3752,7 @@
       </c>
       <c r="D95" s="2"/>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4">
       <c r="A96" s="2">
         <v>95</v>
       </c>
@@ -3526,7 +3764,7 @@
       </c>
       <c r="D96" s="2"/>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4">
       <c r="A97" s="2">
         <v>96</v>
       </c>
@@ -3538,7 +3776,7 @@
       </c>
       <c r="D97" s="2"/>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4">
       <c r="A98" s="2">
         <v>97</v>
       </c>
@@ -3550,7 +3788,7 @@
       </c>
       <c r="D98" s="2"/>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4">
       <c r="A99" s="2">
         <v>98</v>
       </c>
@@ -3562,7 +3800,7 @@
       </c>
       <c r="D99" s="2"/>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4">
       <c r="A100" s="2">
         <v>99</v>
       </c>
@@ -3574,7 +3812,7 @@
       </c>
       <c r="D100" s="2"/>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4">
       <c r="A101" s="2">
         <v>100</v>
       </c>
@@ -3586,25 +3824,25 @@
       </c>
       <c r="D101" s="2"/>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4">
       <c r="A103" s="7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B103" s="7">
         <v>2</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4">
       <c r="A104" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B104" s="7">
         <v>85</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4">
       <c r="A105" s="7" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B105" s="7">
         <v>26</v>
@@ -3621,36 +3859,36 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:D39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="1" max="1" width="22" style="8" customWidth="1"/>
+    <col min="2" max="3" width="18" style="8" customWidth="1"/>
+    <col min="4" max="4" width="12" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18.75" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -3662,7 +3900,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -3674,7 +3912,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -3686,7 +3924,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -3698,7 +3936,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -3710,7 +3948,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -3724,7 +3962,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -3736,7 +3974,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -3748,7 +3986,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -3760,7 +3998,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -3772,7 +4010,7 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -3784,7 +4022,7 @@
       </c>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -3796,7 +4034,7 @@
       </c>
       <c r="D14" s="2"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -3808,7 +4046,7 @@
       </c>
       <c r="D15" s="2"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -3820,7 +4058,7 @@
       </c>
       <c r="D16" s="2"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -3832,7 +4070,7 @@
       </c>
       <c r="D17" s="2"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -3844,7 +4082,7 @@
       </c>
       <c r="D18" s="2"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -3856,7 +4094,7 @@
       </c>
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -3868,7 +4106,7 @@
       </c>
       <c r="D20" s="2"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -3880,7 +4118,7 @@
       </c>
       <c r="D21" s="2"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -3892,7 +4130,7 @@
       </c>
       <c r="D22" s="2"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -3904,7 +4142,7 @@
       </c>
       <c r="D23" s="2"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -3916,7 +4154,7 @@
       </c>
       <c r="D24" s="2"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -3928,7 +4166,7 @@
       </c>
       <c r="D25" s="2"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -3940,7 +4178,7 @@
       </c>
       <c r="D26" s="2"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -3952,7 +4190,7 @@
       </c>
       <c r="D27" s="2"/>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -3964,7 +4202,7 @@
       </c>
       <c r="D28" s="2"/>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -3976,7 +4214,7 @@
       </c>
       <c r="D29" s="2"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -3988,7 +4226,7 @@
       </c>
       <c r="D30" s="2"/>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -4000,7 +4238,7 @@
       </c>
       <c r="D31" s="2"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -4012,7 +4250,7 @@
       </c>
       <c r="D32" s="2"/>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -4024,7 +4262,7 @@
       </c>
       <c r="D33" s="2"/>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -4036,7 +4274,7 @@
       </c>
       <c r="D34" s="2"/>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -4048,25 +4286,25 @@
       </c>
       <c r="D35" s="2"/>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4">
       <c r="A37" s="7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B37" s="7">
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4">
       <c r="A38" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B38" s="7">
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4">
       <c r="A39" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B39" s="7">
         <v>7</v>
@@ -4083,36 +4321,36 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:D26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="1" max="1" width="22" style="8" customWidth="1"/>
+    <col min="2" max="3" width="18" style="8" customWidth="1"/>
+    <col min="4" max="4" width="12" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18.75" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -4124,7 +4362,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -4136,7 +4374,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -4150,7 +4388,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -4162,7 +4400,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -4174,7 +4412,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -4186,7 +4424,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -4198,7 +4436,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -4210,7 +4448,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -4222,7 +4460,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -4234,7 +4472,7 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -4246,7 +4484,7 @@
       </c>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -4258,7 +4496,7 @@
       </c>
       <c r="D14" s="2"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -4270,7 +4508,7 @@
       </c>
       <c r="D15" s="2"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -4282,7 +4520,7 @@
       </c>
       <c r="D16" s="2"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -4294,7 +4532,7 @@
       </c>
       <c r="D17" s="2"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -4306,7 +4544,7 @@
       </c>
       <c r="D18" s="2"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -4318,7 +4556,7 @@
       </c>
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -4330,7 +4568,7 @@
       </c>
       <c r="D20" s="2"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -4342,7 +4580,7 @@
       </c>
       <c r="D21" s="2"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -4354,25 +4592,25 @@
       </c>
       <c r="D22" s="2"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4">
       <c r="A24" s="7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B24" s="7">
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4">
       <c r="A25" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B25" s="7">
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4">
       <c r="A26" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B26" s="7">
         <v>4</v>
@@ -4389,36 +4627,36 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="1" max="1" width="22" style="8" customWidth="1"/>
+    <col min="2" max="3" width="18" style="8" customWidth="1"/>
+    <col min="4" max="4" width="12" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18.75" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -4430,7 +4668,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -4444,7 +4682,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -4456,7 +4694,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -4468,7 +4706,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -4480,7 +4718,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -4492,7 +4730,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -4504,7 +4742,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -4516,25 +4754,25 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4">
       <c r="A12" s="7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B12" s="7">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4">
       <c r="A13" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B13" s="7">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4">
       <c r="A14" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B14" s="7">
         <v>3</v>

</xml_diff>